<commit_message>
ci: fix hardcoded path in generate_vulnerability_excel.js
</commit_message>
<xml_diff>
--- a/Vulnerability_Testing_Report.xlsx
+++ b/Vulnerability_Testing_Report.xlsx
@@ -32,7 +32,7 @@
     <t>PantryWise – Vulnerability Testing Report</t>
   </si>
   <si>
-    <t>Generated: 26/7/2026, 5:09:29 pm  |  Total Test Cases: 420  |  Overall Pass Rate: 100%</t>
+    <t>Generated: 26/7/2026, 5:16:10 pm  |  Total Test Cases: 420  |  Overall Pass Rate: 100%</t>
   </si>
   <si>
     <t>#</t>
@@ -116,7 +116,7 @@
     <t>PantryWise – Vulnerability Testing | All 420 Test Case Names</t>
   </si>
   <si>
-    <t>Generated: 26/7/2026, 5:09:29 pm   |   Total: 420 Test Cases   |   Pass Rate: 100%</t>
+    <t>Generated: 26/7/2026, 5:16:10 pm   |   Total: 420 Test Cases   |   Pass Rate: 100%</t>
   </si>
   <si>
     <t>TC #</t>

</xml_diff>